<commit_message>
tabela de exemplo atualizada
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="16">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -310,8 +310,8 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>45891</v>
@@ -324,8 +324,8 @@
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>45891</v>
@@ -338,8 +338,8 @@
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B4" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>45891</v>
@@ -352,8 +352,8 @@
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B5" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>45891</v>
@@ -366,8 +366,8 @@
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>45891</v>
@@ -380,8 +380,8 @@
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B7" s="1" t="s">
+        <v>1</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>45891</v>

</xml_diff>

<commit_message>
atualização de segurança tabela
</commit_message>
<xml_diff>
--- a/clientes.xlsx
+++ b/clientes.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="17">
   <si>
     <t xml:space="preserve">Nome</t>
   </si>
@@ -35,6 +35,9 @@
   </si>
   <si>
     <t xml:space="preserve">Felipe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">exemple phone</t>
   </si>
   <si>
     <t xml:space="preserve">134,50</t>
@@ -310,84 +313,84 @@
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="n">
-        <v>5551989824424</v>
+      <c r="B2" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>5551989824424</v>
+        <v>7</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="1" t="n">
-        <v>5551989824424</v>
+        <v>9</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C4" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="1" t="n">
-        <v>5551989824424</v>
+        <v>11</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C5" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" s="1" t="n">
-        <v>5551989824424</v>
+        <v>13</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C6" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B7" s="1" t="n">
-        <v>5551989824424</v>
+        <v>15</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>5</v>
       </c>
       <c r="C7" s="2" t="n">
         <v>45891</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>